<commit_message>
feat: agregar modelo de liquidez para Línea de Crédito (LC)
Implementar el flujo completo de cálculo, procesamiento y guardado del modelo Línea de Crédito, incluyendo nuevas rutas de archivos, parámetros y funciones específicas para LC.

Actualiza archivo de parámetros y configuración para soportar la nueva funcionalidad.
</commit_message>
<xml_diff>
--- a/RF_Modelo_Linea_de_Credito/parametros/parametros_ml_lc.xlsx
+++ b/RF_Modelo_Linea_de_Credito/parametros/parametros_ml_lc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmunozb\OneDrive - Falabella\LOCAL_RF\LABS\bfa-cl-modelos-diarios\RF_Modelo_Linea_de_Credito\parametros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45DBA1DE-CF26-4BC0-8A6F-CC148C2B20A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6CF293C-BB61-40C7-9A78-C206919B70B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-14310" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{8BA41A63-8BD0-4DC4-8E7A-ADB7036E65D7}"/>
+    <workbookView xWindow="-120" yWindow="-16590" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8BA41A63-8BD0-4DC4-8E7A-ADB7036E65D7}"/>
   </bookViews>
   <sheets>
     <sheet name="FACTORES" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="46">
   <si>
     <t>CLP</t>
   </si>
@@ -67,15 +67,125 @@
   </si>
   <si>
     <t>DECAY_RATE_ACURRACY</t>
+  </si>
+  <si>
+    <t>CODIGO_EMPRESA</t>
+  </si>
+  <si>
+    <t>OPERACION</t>
+  </si>
+  <si>
+    <t>MONEDA_ORIGEN</t>
+  </si>
+  <si>
+    <t>MONEDA_COMPENSACION</t>
+  </si>
+  <si>
+    <t>COMPENSACION</t>
+  </si>
+  <si>
+    <t>CODIGO_PRODUCTO</t>
+  </si>
+  <si>
+    <t>CODIGO_SUBPRODUCTO</t>
+  </si>
+  <si>
+    <t>NUMERO_CUOTA</t>
+  </si>
+  <si>
+    <t>FECHA_INICIO_CUOTA</t>
+  </si>
+  <si>
+    <t>FECHA_VENCIMIENTO_CUOTA</t>
+  </si>
+  <si>
+    <t>FECHA_REPRICING</t>
+  </si>
+  <si>
+    <t>AMORTIZACION</t>
+  </si>
+  <si>
+    <t>INTERES</t>
+  </si>
+  <si>
+    <t>INTERES_DEVENGADO</t>
+  </si>
+  <si>
+    <t>VP_AMORTIZACION</t>
+  </si>
+  <si>
+    <t>VP_INTERES</t>
+  </si>
+  <si>
+    <t>TIPO_CUOTA</t>
+  </si>
+  <si>
+    <t>CODIGO_ESTRATEGIA</t>
+  </si>
+  <si>
+    <t>CLASIFICACION_CONTABLE</t>
+  </si>
+  <si>
+    <t>INDEXADOR</t>
+  </si>
+  <si>
+    <t>TASA</t>
+  </si>
+  <si>
+    <t>SPREAD</t>
+  </si>
+  <si>
+    <t>PAS</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>ML_C46_Linea_de_Credito_Egreso_Ajustado</t>
+  </si>
+  <si>
+    <t>BALANCE TASAS</t>
+  </si>
+  <si>
+    <t>HTM</t>
+  </si>
+  <si>
+    <t>FECHA_PROCESO</t>
+  </si>
+  <si>
+    <t>COD_ACT/PAS</t>
+  </si>
+  <si>
+    <t>FECHA_CREACION</t>
+  </si>
+  <si>
+    <t>FECHA_PAGO</t>
+  </si>
+  <si>
+    <t>FACTOR_DE_RIESGO</t>
+  </si>
+  <si>
+    <t>AREA_NEGOCIO</t>
+  </si>
+  <si>
+    <t>CODIGO_EJECUTIVO</t>
+  </si>
+  <si>
+    <t>TIPO_TASA</t>
+  </si>
+  <si>
+    <t>TASA_CF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="172" formatCode="_ * #,##0.00000000_ ;_ * \-#,##0.00000000_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00000000_ ;_ * \-#,##0.00000000_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -101,7 +211,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -111,6 +221,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -124,18 +246,54 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="41" fontId="0" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
+    <cellStyle name="Millares" xfId="2" builtinId="3"/>
     <cellStyle name="Millares [0]" xfId="1" builtinId="6"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentaje" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -537,9 +695,863 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63686B3-E724-43F4-B6FB-451FED8CE1B1}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:AE15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="37.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="5" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="7.36328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="O1" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" t="s">
+        <v>41</v>
+      </c>
+      <c r="V1" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="W1" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="X1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y1" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AC1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A2" s="11"/>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="12"/>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="20">
+        <v>314349.05377197301</v>
+      </c>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="22"/>
+      <c r="V2">
+        <v>1</v>
+      </c>
+      <c r="W2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA2">
+        <v>1</v>
+      </c>
+      <c r="AD2" s="17"/>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A3" s="11"/>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K3" s="12"/>
+      <c r="L3">
+        <v>2</v>
+      </c>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="20">
+        <v>154089852.97312903</v>
+      </c>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="22"/>
+      <c r="V3">
+        <v>1</v>
+      </c>
+      <c r="W3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA3">
+        <v>1</v>
+      </c>
+      <c r="AD3" s="17"/>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A4" s="11"/>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" s="12"/>
+      <c r="L4">
+        <v>3</v>
+      </c>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="20">
+        <v>248428379.16703796</v>
+      </c>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="22"/>
+      <c r="V4">
+        <v>1</v>
+      </c>
+      <c r="W4" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA4">
+        <v>1</v>
+      </c>
+      <c r="AD4" s="17"/>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A5" s="11"/>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="12"/>
+      <c r="L5">
+        <v>4</v>
+      </c>
+      <c r="M5" s="12"/>
+      <c r="N5" s="12"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="20">
+        <v>249103182.50524902</v>
+      </c>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="22"/>
+      <c r="V5">
+        <v>1</v>
+      </c>
+      <c r="W5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA5">
+        <v>1</v>
+      </c>
+      <c r="AD5" s="17"/>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A6" s="11"/>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="12"/>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="20">
+        <v>176951094.69189501</v>
+      </c>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="22"/>
+      <c r="V6">
+        <v>1</v>
+      </c>
+      <c r="W6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA6">
+        <v>1</v>
+      </c>
+      <c r="AD6" s="17"/>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A7" s="11"/>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>34</v>
+      </c>
+      <c r="K7" s="12"/>
+      <c r="L7">
+        <v>6</v>
+      </c>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="20">
+        <v>197439324.90778697</v>
+      </c>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="22"/>
+      <c r="V7">
+        <v>1</v>
+      </c>
+      <c r="W7" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA7">
+        <v>1</v>
+      </c>
+      <c r="AD7" s="17"/>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A8" s="11"/>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" t="s">
+        <v>34</v>
+      </c>
+      <c r="K8" s="12"/>
+      <c r="L8">
+        <v>7</v>
+      </c>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="20">
+        <v>273189648.43090999</v>
+      </c>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="22"/>
+      <c r="V8">
+        <v>1</v>
+      </c>
+      <c r="W8" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA8">
+        <v>1</v>
+      </c>
+      <c r="AD8" s="17"/>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A9" s="11"/>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" t="s">
+        <v>34</v>
+      </c>
+      <c r="K9" s="12"/>
+      <c r="L9">
+        <v>14</v>
+      </c>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="20">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="22"/>
+      <c r="V9">
+        <v>1</v>
+      </c>
+      <c r="W9" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA9">
+        <v>1</v>
+      </c>
+      <c r="AD9" s="17"/>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A10" s="11"/>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F10" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10" t="s">
+        <v>34</v>
+      </c>
+      <c r="K10" s="12"/>
+      <c r="L10">
+        <v>28</v>
+      </c>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="20">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="22"/>
+      <c r="V10">
+        <v>1</v>
+      </c>
+      <c r="W10" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA10">
+        <v>1</v>
+      </c>
+      <c r="AD10" s="17"/>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A11" s="11"/>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H11" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" t="s">
+        <v>34</v>
+      </c>
+      <c r="K11" s="12"/>
+      <c r="L11">
+        <v>59</v>
+      </c>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="20">
+        <v>1284743996.8568249</v>
+      </c>
+      <c r="Q11" s="21"/>
+      <c r="R11" s="22"/>
+      <c r="V11">
+        <v>1</v>
+      </c>
+      <c r="W11" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA11">
+        <v>1</v>
+      </c>
+      <c r="AD11" s="17"/>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A12" s="11"/>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F12" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G12" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I12" t="s">
+        <v>34</v>
+      </c>
+      <c r="K12" s="12"/>
+      <c r="L12">
+        <v>89</v>
+      </c>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="20">
+        <v>1952124870.1309502</v>
+      </c>
+      <c r="Q12" s="21"/>
+      <c r="R12" s="22"/>
+      <c r="V12">
+        <v>1</v>
+      </c>
+      <c r="W12" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA12">
+        <v>1</v>
+      </c>
+      <c r="AD12" s="17"/>
+    </row>
+    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A13" s="11"/>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G13" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" t="s">
+        <v>34</v>
+      </c>
+      <c r="I13" t="s">
+        <v>34</v>
+      </c>
+      <c r="K13" s="12"/>
+      <c r="L13">
+        <v>179</v>
+      </c>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="20">
+        <v>4497866508.661869</v>
+      </c>
+      <c r="Q13" s="21"/>
+      <c r="R13" s="22"/>
+      <c r="V13">
+        <v>1</v>
+      </c>
+      <c r="W13" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA13">
+        <v>1</v>
+      </c>
+      <c r="AD13" s="17"/>
+    </row>
+    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A14" s="11"/>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G14" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H14" t="s">
+        <v>34</v>
+      </c>
+      <c r="I14" t="s">
+        <v>34</v>
+      </c>
+      <c r="K14" s="12"/>
+      <c r="L14">
+        <v>350</v>
+      </c>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="20">
+        <v>14426223494.511419</v>
+      </c>
+      <c r="Q14" s="21"/>
+      <c r="R14" s="22"/>
+      <c r="V14">
+        <v>1</v>
+      </c>
+      <c r="W14" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA14">
+        <v>1</v>
+      </c>
+      <c r="AD14" s="17"/>
+    </row>
+    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A15" s="11"/>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G15" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" t="s">
+        <v>34</v>
+      </c>
+      <c r="L15">
+        <v>525</v>
+      </c>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="20">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="21"/>
+      <c r="R15" s="22"/>
+      <c r="V15">
+        <v>1</v>
+      </c>
+      <c r="W15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>35</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA15">
+        <v>1</v>
+      </c>
+      <c r="AD15" s="17"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reescritura mr_prepago_cmr.py para homologar al modelo productivo actual
</commit_message>
<xml_diff>
--- a/RF_Modelo_Linea_de_Credito/parametros/parametros_ml_lc.xlsx
+++ b/RF_Modelo_Linea_de_Credito/parametros/parametros_ml_lc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmunozb\OneDrive - Falabella\LOCAL_RF\LABS\bfa-cl-modelos-diarios\RF_Modelo_Linea_de_Credito\parametros\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vlandaetat\code\bfa-cl-modelos-diarios\RF_Modelo_Linea_de_Credito\parametros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F4A6864-FEB3-4278-8DD3-A9284CF50A6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CF2F02-C1EF-4B3A-92FF-FBD5426ED560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-14790" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8BA41A63-8BD0-4DC4-8E7A-ADB7036E65D7}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8BA41A63-8BD0-4DC4-8E7A-ADB7036E65D7}"/>
   </bookViews>
   <sheets>
     <sheet name="FACTORES" sheetId="4" r:id="rId1"/>
@@ -259,7 +259,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -284,6 +284,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -849,7 +850,7 @@
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="9">
-        <v>314349.05377197301</v>
+        <v>317259.82420349121</v>
       </c>
       <c r="Q2" s="10"/>
       <c r="R2" s="11"/>
@@ -899,7 +900,7 @@
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
       <c r="P3" s="9">
-        <v>154089852.97312903</v>
+        <v>714125244.5105896</v>
       </c>
       <c r="Q3" s="10"/>
       <c r="R3" s="11"/>
@@ -949,7 +950,7 @@
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
       <c r="P4" s="9">
-        <v>248428379.16703796</v>
+        <v>440651271.12638903</v>
       </c>
       <c r="Q4" s="10"/>
       <c r="R4" s="11"/>
@@ -999,7 +1000,7 @@
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
       <c r="P5" s="9">
-        <v>249103182.50524902</v>
+        <v>381182083.85049391</v>
       </c>
       <c r="Q5" s="10"/>
       <c r="R5" s="11"/>
@@ -1049,7 +1050,7 @@
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
       <c r="P6" s="9">
-        <v>176951094.69189501</v>
+        <v>299338842.97463989</v>
       </c>
       <c r="Q6" s="10"/>
       <c r="R6" s="11"/>
@@ -1099,7 +1100,7 @@
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
       <c r="P7" s="9">
-        <v>197439324.90778697</v>
+        <v>178260159.40904212</v>
       </c>
       <c r="Q7" s="10"/>
       <c r="R7" s="11"/>
@@ -1149,7 +1150,7 @@
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
       <c r="P8" s="9">
-        <v>273189648.43090999</v>
+        <v>126577193.88203502</v>
       </c>
       <c r="Q8" s="10"/>
       <c r="R8" s="11"/>
@@ -1199,7 +1200,7 @@
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
       <c r="P9" s="9">
-        <v>0</v>
+        <v>689163108.44747877</v>
       </c>
       <c r="Q9" s="10"/>
       <c r="R9" s="11"/>
@@ -1299,7 +1300,7 @@
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
       <c r="P11" s="9">
-        <v>1284743996.8568249</v>
+        <v>905458052.40490723</v>
       </c>
       <c r="Q11" s="10"/>
       <c r="R11" s="11"/>
@@ -1349,7 +1350,7 @@
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
       <c r="P12" s="9">
-        <v>1952124870.1309502</v>
+        <v>1802951102.3005519</v>
       </c>
       <c r="Q12" s="10"/>
       <c r="R12" s="11"/>
@@ -1399,7 +1400,7 @@
       <c r="N13" s="4"/>
       <c r="O13" s="4"/>
       <c r="P13" s="9">
-        <v>4497866508.661869</v>
+        <v>5203979269.4284668</v>
       </c>
       <c r="Q13" s="10"/>
       <c r="R13" s="11"/>
@@ -1449,9 +1450,9 @@
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
       <c r="P14" s="9">
-        <v>14426223494.511419</v>
-      </c>
-      <c r="Q14" s="10"/>
+        <v>13000892358.669239</v>
+      </c>
+      <c r="Q14" s="16"/>
       <c r="R14" s="11"/>
       <c r="V14">
         <v>1</v>

</xml_diff>

<commit_message>
chore(ml_lc): actualizacion mensual de parametros del modelo
</commit_message>
<xml_diff>
--- a/RF_Modelo_Linea_de_Credito/parametros/parametros_ml_lc.xlsx
+++ b/RF_Modelo_Linea_de_Credito/parametros/parametros_ml_lc.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vlandaetat\code\bfa-cl-modelos-diarios\RF_Modelo_Linea_de_Credito\parametros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CF2F02-C1EF-4B3A-92FF-FBD5426ED560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1551C6-89B9-477C-AA40-3698C833532B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8BA41A63-8BD0-4DC4-8E7A-ADB7036E65D7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{8BA41A63-8BD0-4DC4-8E7A-ADB7036E65D7}"/>
   </bookViews>
   <sheets>
     <sheet name="FACTORES" sheetId="4" r:id="rId1"/>
@@ -233,23 +233,41 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -259,7 +277,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -275,16 +293,18 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="41" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="0" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="0" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="41" fontId="0" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -622,6 +642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D644C8FC-6702-475F-81EF-E45A67C039E0}">
+  <sheetPr codeName="Hoja1"/>
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -692,6 +713,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63686B3-E724-43F4-B6FB-451FED8CE1B1}">
+  <sheetPr codeName="Hoja2"/>
   <dimension ref="A1:AF15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -726,7 +748,7 @@
     <col min="32" max="32" width="28.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>36</v>
       </c>
@@ -751,13 +773,13 @@
       <c r="H1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="13" t="s">
         <v>17</v>
       </c>
       <c r="L1" s="3" t="s">
@@ -772,10 +794,10 @@
       <c r="O1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="P1" s="15" t="s">
+      <c r="P1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="Q1" s="10" t="s">
+      <c r="Q1" s="9" t="s">
         <v>22</v>
       </c>
       <c r="R1" t="s">
@@ -820,7 +842,7 @@
       <c r="AE1" t="s">
         <v>31</v>
       </c>
-      <c r="AF1" s="12" t="s">
+      <c r="AF1" s="11" t="s">
         <v>45</v>
       </c>
     </row>
@@ -849,11 +871,11 @@
       <c r="M2" s="4"/>
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
-      <c r="P2" s="9">
-        <v>317259.82420349121</v>
-      </c>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="11"/>
+      <c r="P2" s="16">
+        <v>318124.48573303223</v>
+      </c>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="10"/>
       <c r="V2">
         <v>1</v>
       </c>
@@ -899,11 +921,11 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
-      <c r="P3" s="9">
-        <v>714125244.5105896</v>
-      </c>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="11"/>
+      <c r="P3" s="17">
+        <v>1416777693.374115</v>
+      </c>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="10"/>
       <c r="V3">
         <v>1</v>
       </c>
@@ -949,11 +971,11 @@
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
-      <c r="P4" s="9">
-        <v>440651271.12638903</v>
-      </c>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="11"/>
+      <c r="P4" s="17">
+        <v>471790916.24951196</v>
+      </c>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="10"/>
       <c r="V4">
         <v>1</v>
       </c>
@@ -999,11 +1021,11 @@
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
-      <c r="P5" s="9">
-        <v>381182083.85049391</v>
-      </c>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="11"/>
+      <c r="P5" s="17">
+        <v>305877952.6179502</v>
+      </c>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="10"/>
       <c r="V5">
         <v>1</v>
       </c>
@@ -1049,11 +1071,11 @@
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
-      <c r="P6" s="9">
-        <v>299338842.97463989</v>
-      </c>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="11"/>
+      <c r="P6" s="17">
+        <v>161855907.92533875</v>
+      </c>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="10"/>
       <c r="V6">
         <v>1</v>
       </c>
@@ -1099,11 +1121,11 @@
       <c r="M7" s="4"/>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
-      <c r="P7" s="9">
-        <v>178260159.40904212</v>
-      </c>
-      <c r="Q7" s="10"/>
-      <c r="R7" s="11"/>
+      <c r="P7" s="17">
+        <v>130187875.54225206</v>
+      </c>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="10"/>
       <c r="V7">
         <v>1</v>
       </c>
@@ -1149,11 +1171,11 @@
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
-      <c r="P8" s="9">
-        <v>126577193.88203502</v>
-      </c>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="11"/>
+      <c r="P8" s="17">
+        <v>277824964.70605421</v>
+      </c>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="10"/>
       <c r="V8">
         <v>1</v>
       </c>
@@ -1199,11 +1221,11 @@
       <c r="M9" s="4"/>
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
-      <c r="P9" s="9">
-        <v>689163108.44747877</v>
-      </c>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="11"/>
+      <c r="P9" s="17">
+        <v>582710116.8488307</v>
+      </c>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="10"/>
       <c r="V9">
         <v>1</v>
       </c>
@@ -1249,11 +1271,11 @@
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
-      <c r="P10" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="11"/>
+      <c r="P10" s="17">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="10"/>
       <c r="V10">
         <v>1</v>
       </c>
@@ -1299,11 +1321,11 @@
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
-      <c r="P11" s="9">
-        <v>905458052.40490723</v>
-      </c>
-      <c r="Q11" s="10"/>
-      <c r="R11" s="11"/>
+      <c r="P11" s="17">
+        <v>833649686.90783691</v>
+      </c>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="10"/>
       <c r="V11">
         <v>1</v>
       </c>
@@ -1349,11 +1371,11 @@
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
-      <c r="P12" s="9">
-        <v>1802951102.3005519</v>
-      </c>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="11"/>
+      <c r="P12" s="17">
+        <v>1354208104.4548798</v>
+      </c>
+      <c r="Q12" s="9"/>
+      <c r="R12" s="10"/>
       <c r="V12">
         <v>1</v>
       </c>
@@ -1399,11 +1421,11 @@
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
       <c r="O13" s="4"/>
-      <c r="P13" s="9">
-        <v>5203979269.4284668</v>
-      </c>
-      <c r="Q13" s="10"/>
-      <c r="R13" s="11"/>
+      <c r="P13" s="17">
+        <v>5263214932.5449371</v>
+      </c>
+      <c r="Q13" s="9"/>
+      <c r="R13" s="10"/>
       <c r="V13">
         <v>1</v>
       </c>
@@ -1449,11 +1471,11 @@
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
       <c r="O14" s="4"/>
-      <c r="P14" s="9">
-        <v>13000892358.669239</v>
-      </c>
-      <c r="Q14" s="16"/>
-      <c r="R14" s="11"/>
+      <c r="P14" s="17">
+        <v>12482453027.902985</v>
+      </c>
+      <c r="Q14" s="15"/>
+      <c r="R14" s="10"/>
       <c r="V14">
         <v>1</v>
       </c>
@@ -1474,7 +1496,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3"/>
       <c r="B15">
         <v>1</v>
@@ -1498,11 +1520,11 @@
       <c r="M15" s="4"/>
       <c r="N15" s="4"/>
       <c r="O15" s="4"/>
-      <c r="P15" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="10"/>
-      <c r="R15" s="11"/>
+      <c r="P15" s="18">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="9"/>
+      <c r="R15" s="10"/>
       <c r="V15">
         <v>1</v>
       </c>

</xml_diff>